<commit_message>
Adventure hero: wrap multi-image carousels into a carousel block
10 of 16 adventure pages have a source .cmp-carousel hero with 2-3 slides. The
importer was flattening those into stacked <picture> paragraphs, so they rendered
one below the other instead of as a slideshow. In the adventure transformer's
beforeTransform, convert any .cmp-carousel with 2+ images into an EDS carousel
block table (one row per slide). Single-image heroes are left as full-bleed
banners.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-wknd-adventure.report.xlsx
+++ b/tools/importer/reports/import-wknd-adventure.report.xlsx
@@ -607,7 +607,7 @@
     <t>us/en/faqs</t>
   </si>
   <si>
-    <t>2026-08-12T11:10:39.124Z</t>
+    <t>2026-08-12T11:51:45.004Z</t>
   </si>
   <si>
     <t>us/en/magazine.report.json</t>
@@ -634,7 +634,7 @@
     <t>us/en/adventures/bali-surf-camp</t>
   </si>
   <si>
-    <t>2026-08-12T11:13:39.792Z</t>
+    <t>2026-08-13T13:56:20.947Z</t>
   </si>
   <si>
     <t>us/en/adventures/beervana-portland.report.json</t>
@@ -643,7 +643,7 @@
     <t>us/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-08-12T11:13:44.785Z</t>
+    <t>2026-08-13T13:56:25.208Z</t>
   </si>
   <si>
     <t>us/en/adventures/climbing-new-zealand.report.json</t>
@@ -652,7 +652,7 @@
     <t>us/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-08-12T11:13:50.857Z</t>
+    <t>2026-08-13T13:56:30.144Z</t>
   </si>
   <si>
     <t>us/en/adventures/colorado-rock-climbing.report.json</t>
@@ -661,7 +661,7 @@
     <t>us/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-08-12T11:13:56.233Z</t>
+    <t>2026-08-13T13:56:34.346Z</t>
   </si>
   <si>
     <t>us/en/adventures/cycling-southern-utah.report.json</t>
@@ -670,7 +670,7 @@
     <t>us/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-08-12T11:14:01.771Z</t>
+    <t>2026-08-13T13:56:39.594Z</t>
   </si>
   <si>
     <t>us/en/adventures/cycling-tuscany.report.json</t>
@@ -679,7 +679,7 @@
     <t>us/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-08-12T11:14:08.370Z</t>
+    <t>2026-08-13T13:56:44.710Z</t>
   </si>
   <si>
     <t>us/en/adventures/downhill-skiing-wyoming.report.json</t>
@@ -688,7 +688,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-08-12T11:14:14.332Z</t>
+    <t>2026-08-13T13:56:49.961Z</t>
   </si>
   <si>
     <t>us/en/adventures/gastronomic-marais-tour.report.json</t>
@@ -697,7 +697,7 @@
     <t>us/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-08-12T11:14:20.890Z</t>
+    <t>2026-08-13T13:56:55.269Z</t>
   </si>
   <si>
     <t>us/en/adventures/napa-wine-tasting.report.json</t>
@@ -706,7 +706,7 @@
     <t>us/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-08-12T11:14:27.665Z</t>
+    <t>2026-08-13T13:56:59.952Z</t>
   </si>
   <si>
     <t>us/en/adventures/riverside-camping-australia.report.json</t>
@@ -715,7 +715,7 @@
     <t>us/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-08-12T11:14:32.303Z</t>
+    <t>2026-08-13T13:57:04.923Z</t>
   </si>
   <si>
     <t>us/en/adventures/ski-touring-mont-blanc.report.json</t>
@@ -724,7 +724,7 @@
     <t>us/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-08-12T11:14:36.207Z</t>
+    <t>2026-08-13T13:57:08.893Z</t>
   </si>
   <si>
     <t>us/en/adventures/surf-camp-costa-rica.report.json</t>
@@ -733,7 +733,7 @@
     <t>us/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-08-12T11:14:40.687Z</t>
+    <t>2026-08-13T13:57:13.664Z</t>
   </si>
   <si>
     <t>us/en/adventures/tahoe-skiing.report.json</t>
@@ -742,7 +742,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-08-12T11:14:47.245Z</t>
+    <t>2026-08-13T13:57:19.872Z</t>
   </si>
   <si>
     <t>us/en/adventures/west-coast-cycling.report.json</t>
@@ -751,7 +751,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-08-12T11:14:52.150Z</t>
+    <t>2026-08-13T13:57:25.480Z</t>
   </si>
   <si>
     <t>us/en/adventures/whistler-mountain-biking.report.json</t>
@@ -760,7 +760,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-08-12T11:14:57.767Z</t>
+    <t>2026-08-13T13:57:30.131Z</t>
   </si>
   <si>
     <t>us/en/adventures/yosemite-backpacking.html.report.json</t>
@@ -789,7 +789,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-08-12T11:15:01.781Z</t>
+    <t>2026-08-13T13:57:34.057Z</t>
   </si>
   <si>
     <t>us/en/magazine/arctic-surfing.report.json</t>
@@ -798,7 +798,7 @@
     <t>us/en/magazine/arctic-surfing</t>
   </si>
   <si>
-    <t>2026-08-12T11:13:13.925Z</t>
+    <t>2026-08-12T12:45:50.848Z</t>
   </si>
   <si>
     <t>us/en/magazine/guide-la-skateparks.report.json</t>
@@ -807,7 +807,7 @@
     <t>us/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-08-12T11:13:18.992Z</t>
+    <t>2026-08-12T12:45:56.055Z</t>
   </si>
   <si>
     <t>us/en/magazine/san-diego-surf.report.json</t>
@@ -816,7 +816,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-08-12T11:13:25.163Z</t>
+    <t>2026-08-12T12:46:00.979Z</t>
   </si>
   <si>
     <t>us/en/magazine/ski-touring.report.json</t>
@@ -825,7 +825,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-08-12T11:13:30.153Z</t>
+    <t>2026-08-12T12:46:07.398Z</t>
   </si>
   <si>
     <t>us/en/magazine/western-australia.report.json</t>
@@ -834,7 +834,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-08-12T11:13:35.310Z</t>
+    <t>2026-08-12T12:46:11.910Z</t>
   </si>
 </sst>
 </file>

</xml_diff>